<commit_message>
add npm start command
</commit_message>
<xml_diff>
--- a/Techem_Smart_Export_2026-04-13.xlsx
+++ b/Techem_Smart_Export_2026-04-13.xlsx
@@ -1,21 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
-  <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1C15596-C9BF-4D57-BE14-F0D6974D6060}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet name="Verbrauchsübersicht" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="Verbrauchsübersicht" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="12">
   <si>
     <t>Monat</t>
   </si>
@@ -51,82 +47,23 @@
   </si>
   <si>
     <t>2024-06</t>
-  </si>
-  <si>
-    <t>2024-07</t>
-  </si>
-  <si>
-    <t>2024-08</t>
-  </si>
-  <si>
-    <t>2024-09</t>
-  </si>
-  <si>
-    <t>2024-10</t>
-  </si>
-  <si>
-    <t>2024-11</t>
-  </si>
-  <si>
-    <t>2024-12</t>
-  </si>
-  <si>
-    <t>2025-01</t>
-  </si>
-  <si>
-    <t>2025-02</t>
-  </si>
-  <si>
-    <t>2025-03</t>
-  </si>
-  <si>
-    <t>2025-04</t>
-  </si>
-  <si>
-    <t>2025-05</t>
-  </si>
-  <si>
-    <t>2025-06</t>
-  </si>
-  <si>
-    <t>2025-07</t>
-  </si>
-  <si>
-    <t>2025-08</t>
-  </si>
-  <si>
-    <t>2025-09</t>
-  </si>
-  <si>
-    <t>2025-10</t>
-  </si>
-  <si>
-    <t>2025-11</t>
-  </si>
-  <si>
-    <t>2025-12</t>
-  </si>
-  <si>
-    <t>2026-01</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="4">
@@ -508,15 +445,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E26"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="2" max="2" width="27.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="22.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="4" width="25" customWidth="1"/>
+    <col min="5" max="5" width="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -638,332 +575,9 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B8" s="2">
-        <v>14</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D8" s="2">
-        <v>0</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B9" s="3">
-        <v>0</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D9" s="3">
-        <v>0</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B10" s="2">
-        <v>14</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D10" s="2">
-        <v>0</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B11" s="3">
-        <v>0</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D11" s="3">
-        <v>0</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B12" s="2">
-        <v>14</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D12" s="2">
-        <v>81</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="B13" s="3">
-        <v>0</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D13" s="3">
-        <v>45</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B14" s="2">
-        <v>0</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D14" s="2">
-        <v>73</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="B15" s="3">
-        <v>0</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D15" s="3">
-        <v>122</v>
-      </c>
-      <c r="E15" s="3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B16" s="2">
-        <v>14</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D16" s="2">
-        <v>0</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="B17" s="3">
-        <v>6</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D17" s="3">
-        <v>23</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B18" s="2">
-        <v>6</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D18" s="2">
-        <v>13</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="B19" s="3">
-        <v>6</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D19" s="3">
-        <v>0</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B20" s="2">
-        <v>6</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D20" s="2">
-        <v>0</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="B21" s="3">
-        <v>6</v>
-      </c>
-      <c r="C21" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D21" s="3">
-        <v>0</v>
-      </c>
-      <c r="E21" s="3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="B22" s="2">
-        <v>5</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D22" s="2">
-        <v>11</v>
-      </c>
-      <c r="E22" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="B23" s="3">
-        <v>6</v>
-      </c>
-      <c r="C23" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D23" s="3">
-        <v>31</v>
-      </c>
-      <c r="E23" s="3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="B24" s="2">
-        <v>5</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D24" s="2">
-        <v>48</v>
-      </c>
-      <c r="E24" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="B25" s="3">
-        <v>6</v>
-      </c>
-      <c r="C25" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D25" s="3">
-        <v>70</v>
-      </c>
-      <c r="E25" s="3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="B26" s="2">
-        <v>4</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D26" s="2">
-        <v>67</v>
-      </c>
-      <c r="E26" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:E1" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:E1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>